<commit_message>
Atualiza datasets e automacoes
</commit_message>
<xml_diff>
--- a/liga_serie_A/datasets_liga_serie_A/Pontuacoes_Liga_1_Turno_Completa.xlsx
+++ b/liga_serie_A/datasets_liga_serie_A/Pontuacoes_Liga_1_Turno_Completa.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -73,6 +73,9 @@
     <t>Rodada 19</t>
   </si>
   <si>
+    <t>Atlético Colorado 2021</t>
+  </si>
+  <si>
     <t>cartola scheuer17</t>
   </si>
   <si>
@@ -122,6 +125,9 @@
   </si>
   <si>
     <t>TIGRE LEON</t>
+  </si>
+  <si>
+    <t>TORRESMO COM PINGA PRO26.2</t>
   </si>
   <si>
     <t>VASCO MARTINS FC</t>
@@ -485,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -552,7 +558,7 @@
         <v>19</v>
       </c>
       <c r="B2">
-        <v>61.56</v>
+        <v>53.260009765625</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -560,7 +566,7 @@
         <v>20</v>
       </c>
       <c r="B3">
-        <v>72.7</v>
+        <v>61.56005859375</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -568,7 +574,7 @@
         <v>21</v>
       </c>
       <c r="B4">
-        <v>53.66</v>
+        <v>72.7001953125</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -576,7 +582,7 @@
         <v>22</v>
       </c>
       <c r="B5">
-        <v>63.9</v>
+        <v>53.659912109375</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -584,7 +590,7 @@
         <v>23</v>
       </c>
       <c r="B6">
-        <v>57.45</v>
+        <v>63.89990234375</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -592,7 +598,7 @@
         <v>24</v>
       </c>
       <c r="B7">
-        <v>47.86</v>
+        <v>57.449951171875</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -600,7 +606,7 @@
         <v>25</v>
       </c>
       <c r="B8">
-        <v>62.56</v>
+        <v>47.860107421875</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -608,7 +614,7 @@
         <v>26</v>
       </c>
       <c r="B9">
-        <v>58.51</v>
+        <v>62.56005859375</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -616,7 +622,7 @@
         <v>27</v>
       </c>
       <c r="B10">
-        <v>73.95999999999999</v>
+        <v>58.510009765625</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -624,7 +630,7 @@
         <v>28</v>
       </c>
       <c r="B11">
-        <v>84.26000000000001</v>
+        <v>73.9599609375</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -632,7 +638,7 @@
         <v>29</v>
       </c>
       <c r="B12">
-        <v>50.26</v>
+        <v>84.259765625</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -640,7 +646,7 @@
         <v>30</v>
       </c>
       <c r="B13">
-        <v>59.25</v>
+        <v>50.260009765625</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -648,7 +654,7 @@
         <v>31</v>
       </c>
       <c r="B14">
-        <v>60.16</v>
+        <v>59.25</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -656,7 +662,7 @@
         <v>32</v>
       </c>
       <c r="B15">
-        <v>66.86</v>
+        <v>60.159912109375</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -664,7 +670,7 @@
         <v>33</v>
       </c>
       <c r="B16">
-        <v>58.96</v>
+        <v>66.85986328125</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -672,7 +678,7 @@
         <v>34</v>
       </c>
       <c r="B17">
-        <v>68.06</v>
+        <v>58.9599609375</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -680,7 +686,7 @@
         <v>35</v>
       </c>
       <c r="B18">
-        <v>51.26</v>
+        <v>68.06005859375</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -688,15 +694,31 @@
         <v>36</v>
       </c>
       <c r="B19">
-        <v>55.9</v>
+        <v>51.260009765625</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B20" t="s">
-        <v>28</v>
+      <c r="B20">
+        <v>73.759765625</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21">
+        <v>55.89990234375</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>